<commit_message>
docs(tracker,bom): v28 — add bring-up hardware (Actions #32/#33: charge/protection circuit, breadboard+jumper wires, resistor/capacitor assortment); renumber action register to 33 items; fix stale §2.6 locked v27 labels to v28
</commit_message>
<xml_diff>
--- a/docs/SPARK_BOM_Procurement.xlsx
+++ b/docs/SPARK_BOM_Procurement.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="11" min="1" max="1"/>
@@ -524,47 +524,47 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="12">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Unit Price (NPR)</t>
         </is>
       </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>Line Total (NPR)</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>Funding Source</t>
         </is>
       </c>
-      <c r="G1" s="13" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="13" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>Action Ref</t>
         </is>
       </c>
-      <c r="I1" s="13" t="inlineStr">
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -611,7 +611,7 @@
           <t>1 self-funded (Aaradhya) + 1 dept ask</t>
         </is>
       </c>
-      <c r="G3" s="19" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>Ordering pending — Action #16 spare unit not yet added</t>
         </is>
@@ -653,7 +653,7 @@
           <t>Lab-borrowed, no cost</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>Receipt/availability unconfirmed</t>
         </is>
@@ -695,7 +695,7 @@
           <t>Unpriced placeholder</t>
         </is>
       </c>
-      <c r="G5" s="19" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Spec locked v28 (1000 mAh Li-ion/LiPo) — sourcing not started</t>
         </is>
@@ -737,7 +737,7 @@
           <t>Self-funded (Aaradhya), price unlogged</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>Open — price not recorded</t>
         </is>
@@ -756,7 +756,7 @@
     <row r="7" ht="23.85" customHeight="1" s="12">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>Enclosure (3D-printed PLA)</t>
+          <t>Charge/protection circuit (TP4056-class)</t>
         </is>
       </c>
       <c r="B7" s="17" t="n">
@@ -764,11 +764,11 @@
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>KEC Makerspace (in-house)</t>
+          <t>TBD (vendor, baseline SLT Pvt.Ltd)</t>
         </is>
       </c>
       <c r="D7" s="18" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E7" s="18">
         <f>B7*D7</f>
@@ -776,166 +776,345 @@
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
+          <t>Unpriced-baseline (legacy proposal pricing)</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>New v28 — required unless sourced battery is a protected pack</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>#32</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Added v28. Drop this line if the purchased battery cell already includes protection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="12">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Enclosure (3D-printed PLA)</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>KEC Makerspace (in-house)</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="17">
+        <f>B8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
           <t>Material cost negligible; labor in-house</t>
         </is>
       </c>
-      <c r="G7" s="19" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>Method + form factor both resolved — wrist-worn (Action #8, locked v28)</t>
         </is>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
         <is>
           <t>#8, #11</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>Wrist-worn, locked v28. Threshold calibration (Action #7) can proceed against fixed geometry.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="12">
-      <c r="A8" s="14" t="inlineStr">
+    <row r="9" ht="23.85" customHeight="1" s="12">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Gateway</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n"/>
-      <c r="C8" s="15" t="n"/>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="15" t="n"/>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="23.85" customHeight="1" s="12">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="16" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="12">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Acer Swift Go 16 (laptop, already owned)</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B10" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>Owned</t>
         </is>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D10" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="18">
-        <f>B9*D9</f>
+      <c r="E10" s="17">
+        <f>B10*D10</f>
         <v/>
       </c>
-      <c r="F9" s="17" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>No cost</t>
         </is>
       </c>
-      <c r="G9" s="20" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>Resolved — in hand</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>#15</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>Compute sufficiency confirmed vs RPi 4B (v15)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="12">
-      <c r="A10" s="14" t="inlineStr">
+    <row r="11" ht="23.85" customHeight="1" s="12">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="15" t="n"/>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="16" t="n"/>
-    </row>
-    <row r="11" ht="23.85" customHeight="1" s="12">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="16" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>BLE dongle</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B12" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>TBD (vendor)</t>
         </is>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D12" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="18">
-        <f>B11*D11</f>
+      <c r="E12" s="17">
+        <f>B12*D12</f>
         <v/>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>Unpriced</t>
         </is>
       </c>
-      <c r="G11" s="19" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>Modality locked v28 — dongle required (phone app confirmed)</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>Phone app confirmed v28; dongle required over built-in BLE. Vendor/price not yet sourced.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Bring-up/Assembly</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="16" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Breadboard + jumper wires</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>TBD (vendor, baseline SLT Pvt.Ltd)</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>325</v>
+      </c>
+      <c r="E14" s="17">
+        <f>B14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Unpriced-baseline (legacy proposal pricing)</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>New v28 — bring-up/prototyping hardware</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>#33</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>Added v28. 2 sets, per legacy table pricing (NPR 325/set).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="12">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Resistor/capacitor assortment</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>1 lot</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>TBD (vendor, baseline Himalayan Solutions)</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>600</v>
+      </c>
+      <c r="E15" s="17">
+        <f>B15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>Unpriced-baseline (legacy proposal pricing)</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>New v28 — bring-up/prototyping hardware</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>#33</t>
+        </is>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>Added v28. 1 lot, per legacy table pricing (NPR 600/lot).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>TOTAL PROJECT COST</t>
         </is>
       </c>
-      <c r="B13" s="22" t="n"/>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="23">
-        <f>SUM(E2:E11)</f>
+      <c r="B17" s="17" t="n"/>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="17">
+        <f>SUM(E2:E15)</f>
         <v/>
       </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="12">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>Source: dev_logs/SPARK_TRACKER.md §2.6, §1 (Actions #16,#18,#19). Prior confirmed total ~NPR 15,004 (v22/v13).</t>
-        </is>
-      </c>
-    </row>
+      <c r="F17" s="17" t="n"/>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="17" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="17" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Source: dev_logs/SPARK_TRACKER.md §2.6, §1 (Actions #16,#18,#19,#32,#33). Prior confirmed total ~NPR 15,004 (v22/v13); v28 adds ~NPR 1,340 baseline for Actions #32/#33 bring-up hardware.</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="16" t="n"/>
+    </row>
+    <row r="20"/>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A8:I8"/>
+  <mergeCells count="5">
+    <mergeCell ref="A19:I19"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A9:I9"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
docs(tracker,bom): v29 — lock enclosure electronics placement top-of-wrist/dorsal (Action #34); fix stale locked v27 labels in §2.2 and R-05 risk matrix
</commit_message>
<xml_diff>
--- a/docs/SPARK_BOM_Procurement.xlsx
+++ b/docs/SPARK_BOM_Procurement.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="11" min="1" max="1"/>
@@ -828,12 +828,12 @@
       </c>
       <c r="H8" s="17" t="inlineStr">
         <is>
-          <t>#8, #11</t>
+          <t>#8, #11, #34</t>
         </is>
       </c>
       <c r="I8" s="17" t="inlineStr">
         <is>
-          <t>Wrist-worn, locked v28. Threshold calibration (Action #7) can proceed against fixed geometry.</t>
+          <t>Wrist-worn, locked v28. Electronics top-of-wrist/dorsal, locked v29 (Action #34). Threshold calibration (Action #7) can proceed against fixed geometry.</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,6 @@
       <c r="H19" s="15" t="n"/>
       <c r="I19" s="16" t="n"/>
     </row>
-    <row r="20"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A19:I19"/>

</xml_diff>